<commit_message>
ID update on contribution sheet
</commit_message>
<xml_diff>
--- a/Documents/Group7ContributionSheet.xlsx
+++ b/Documents/Group7ContributionSheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BSc Final Module\DevOps\Group7DevOps\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EEBBA24-8D60-4E5C-A9A4-B645A82F1579}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F116403-41E7-46ED-AEA6-0AA2147E4EED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{A2F8506F-6572-4641-9F72-ADE6701B11D3}"/>
   </bookViews>
@@ -68,9 +68,6 @@
     <t>40841064 (Aye Kyawt Moe)</t>
   </si>
   <si>
-    <t>(Inkyin Phyu)</t>
-  </si>
-  <si>
     <t>40841063 (Hlum Htet Aung)</t>
   </si>
   <si>
@@ -78,6 +75,9 @@
   </si>
   <si>
     <t>(Sharma, Paras)</t>
+  </si>
+  <si>
+    <t>40841055 (Inkyin Phyu)</t>
   </si>
 </sst>
 </file>
@@ -566,7 +566,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B7" s="3">
         <v>14.28</v>
@@ -575,7 +575,7 @@
     </row>
     <row r="8" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B8" s="3">
         <v>14.28</v>
@@ -584,7 +584,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B9" s="3">
         <v>14.28</v>
@@ -593,7 +593,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B10" s="4">
         <f>SUM(B3:B9)</f>

</xml_diff>

<commit_message>
Read me badges update
</commit_message>
<xml_diff>
--- a/Documents/Group7ContributionSheet.xlsx
+++ b/Documents/Group7ContributionSheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BSc Final Module\DevOps\Group7DevOps\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F116403-41E7-46ED-AEA6-0AA2147E4EED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{850F2F45-A316-4F5F-B375-3A964EE1576D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{A2F8506F-6572-4641-9F72-ADE6701B11D3}"/>
   </bookViews>
@@ -74,10 +74,10 @@
     <t>Total</t>
   </si>
   <si>
-    <t>(Sharma, Paras)</t>
-  </si>
-  <si>
     <t>40841055 (Inkyin Phyu)</t>
+  </si>
+  <si>
+    <t>(Sharma, Paras) (Absence as of now)</t>
   </si>
 </sst>
 </file>
@@ -566,7 +566,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B7" s="3">
         <v>14.28</v>
@@ -582,9 +582,9 @@
       </c>
       <c r="C8" s="3"/>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B9" s="3">
         <v>14.28</v>

</xml_diff>